<commit_message>
chore(data): fix excessive future dates in seed excel
</commit_message>
<xml_diff>
--- a/rusun-backend/seed_data/Data_Penghuni_Cleaned.xlsx
+++ b/rusun-backend/seed_data/Data_Penghuni_Cleaned.xlsx
@@ -8098,12 +8098,12 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>2028-02-27</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -8674,12 +8674,12 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>2028-02-27</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -11118,12 +11118,12 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>2028-02-24</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J223" t="inlineStr">
@@ -11598,12 +11598,12 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">
@@ -12554,12 +12554,12 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
@@ -13322,12 +13322,12 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
@@ -14138,12 +14138,12 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J286" t="inlineStr">
@@ -14570,12 +14570,12 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J295" t="inlineStr">
@@ -14810,12 +14810,12 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J300" t="inlineStr">
@@ -15050,12 +15050,12 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J305" t="inlineStr">
@@ -15818,12 +15818,12 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J321" t="inlineStr">
@@ -16298,12 +16298,12 @@
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I331" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J331" t="inlineStr">
@@ -16826,12 +16826,12 @@
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I342" t="inlineStr">
         <is>
-          <t>2028-03-12</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J342" t="inlineStr">
@@ -17210,12 +17210,12 @@
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I350" t="inlineStr">
         <is>
-          <t>2028-03-12</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J350" t="inlineStr">
@@ -17402,12 +17402,12 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J354" t="inlineStr">
@@ -17738,12 +17738,12 @@
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I361" t="inlineStr">
         <is>
-          <t>2028-02-04</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J361" t="inlineStr">
@@ -17786,12 +17786,12 @@
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I362" t="inlineStr">
         <is>
-          <t>2028-03-05</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J362" t="inlineStr">
@@ -19510,12 +19510,12 @@
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J398" t="inlineStr">
@@ -22142,12 +22142,12 @@
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I453" t="inlineStr">
         <is>
-          <t>2028-02-06</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J453" t="inlineStr">
@@ -22430,12 +22430,12 @@
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I459" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J459" t="inlineStr">
@@ -23150,12 +23150,12 @@
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I474" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J474" t="inlineStr">
@@ -24206,12 +24206,12 @@
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I496" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J496" t="inlineStr">
@@ -25118,12 +25118,12 @@
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I515" t="inlineStr">
         <is>
-          <t>2028-03-02</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J515" t="inlineStr"/>
@@ -26410,12 +26410,12 @@
       </c>
       <c r="H542" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I542" t="inlineStr">
         <is>
-          <t>2028-02-05</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J542" t="inlineStr">
@@ -26602,12 +26602,12 @@
       </c>
       <c r="H546" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I546" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J546" t="inlineStr">
@@ -28222,12 +28222,12 @@
       </c>
       <c r="H580" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I580" t="inlineStr">
         <is>
-          <t>2028-04-02</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J580" t="inlineStr"/>
@@ -28458,12 +28458,12 @@
       </c>
       <c r="H585" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I585" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J585" t="inlineStr"/>
@@ -28838,12 +28838,12 @@
       </c>
       <c r="H593" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I593" t="inlineStr">
         <is>
-          <t>2028-02-12</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J593" t="inlineStr">
@@ -29222,12 +29222,12 @@
       </c>
       <c r="H601" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I601" t="inlineStr">
         <is>
-          <t>2028-02-11</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J601" t="inlineStr">
@@ -29414,12 +29414,12 @@
       </c>
       <c r="H605" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I605" t="inlineStr">
         <is>
-          <t>2028-03-02</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J605" t="inlineStr">
@@ -30082,12 +30082,12 @@
       </c>
       <c r="H619" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I619" t="inlineStr">
         <is>
-          <t>2028-04-09</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J619" t="inlineStr"/>
@@ -30266,12 +30266,12 @@
       </c>
       <c r="H623" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I623" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J623" t="inlineStr">
@@ -31442,12 +31442,12 @@
       </c>
       <c r="H648" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I648" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J648" t="inlineStr">
@@ -31634,12 +31634,12 @@
       </c>
       <c r="H652" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I652" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J652" t="inlineStr">
@@ -34014,12 +34014,12 @@
       </c>
       <c r="H702" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I702" t="inlineStr">
         <is>
-          <t>2028-02-12</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J702" t="inlineStr">
@@ -36958,12 +36958,12 @@
       </c>
       <c r="H764" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I764" t="inlineStr">
         <is>
-          <t>2028-04-10</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="J764" t="inlineStr"/>

</xml_diff>